<commit_message>
Edited the search querry
</commit_message>
<xml_diff>
--- a/leads_crm.xlsx
+++ b/leads_crm.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7BA5E20-54A2-494B-8847-2BD4D667096A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Qualified Leads" state="visible" r:id="rId4"/>
+    <sheet name="Qualified Leads" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -79,60 +83,39 @@
     <t>📲 Send Message</t>
   </si>
   <si>
-    <t>Hello Fuzion Salon &amp; Spa team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
-  </si>
-  <si>
     <t>Kauser beauty parlour</t>
   </si>
   <si>
     <t>No Phone</t>
   </si>
   <si>
-    <t>Hello Kauser beauty parlour team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
-  </si>
-  <si>
     <t>𝐁𝐞𝐚𝐮𝐭𝐲 𝐂𝐚𝐫𝐞 𝐛𝐲 𝐍𝐚𝐛𝐢𝐥𝐚 (Gulberg Branch)</t>
   </si>
   <si>
     <t>Phone: +92 42 37897908</t>
   </si>
   <si>
-    <t>Hello 𝐁𝐞𝐚𝐮𝐭𝐲 𝐂𝐚𝐫𝐞 𝐛𝐲 𝐍𝐚𝐛𝐢𝐥𝐚 (Gulberg Branch) team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
-  </si>
-  <si>
     <t>Beauty Icon Salon, Makeup Lounge &amp; Ladies GYM</t>
   </si>
   <si>
-    <t>Hello Beauty Icon Salon, Makeup Lounge &amp; Ladies GYM team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
-  </si>
-  <si>
     <t>Beauty Queen Beauty Parlour</t>
   </si>
   <si>
     <t>Phone: +92 324 4585814</t>
   </si>
   <si>
-    <t>Hello Beauty Queen Beauty Parlour team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
-  </si>
-  <si>
     <t>Shimla Beauty Parlor - Hair Salon Best beauty parlor in Lahore</t>
   </si>
   <si>
     <t>Phone: +92 300 4990519</t>
   </si>
   <si>
-    <t>Hello Shimla Beauty Parlor - Hair Salon Best beauty parlor in Lahore team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
-  </si>
-  <si>
     <t>Hamna's Beauty salon &amp; Bridal Studio</t>
   </si>
   <si>
     <t>Phone: +92 42 35170702</t>
   </si>
   <si>
-    <t>Hello Hamna's Beauty salon &amp; Bridal Studio team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
-  </si>
-  <si>
     <t>Needs Redesign/Audit</t>
   </si>
   <si>
@@ -175,9 +158,6 @@
     <t>❌ No</t>
   </si>
   <si>
-    <t>Hello Shafaq n Kami salon | Best Salon &amp; Studio in Lahore, Pakistan team! I love what you guys are building. I noticed you are currently running paid ads, but your website takes a massive 6.8 seconds to load. You are paying for traffic but likely losing customers to slow load times before they see your products. I built a high-speed React prototype for you that loads instantly with a 1-click WhatsApp checkout. Check it out here: https://pkgarments-demo.netlify.app/ Let me know what you think!</t>
-  </si>
-  <si>
     <t>screenshots/Shafaq_n_Kami_salon___Best_Salon___Studio_in_Lahore__Pakistan.png</t>
   </si>
   <si>
@@ -193,9 +173,6 @@
     <t>28.3s</t>
   </si>
   <si>
-    <t>Hello CANVAS Salon Lahore | Best Hair and Bridal Parlour Gulberg team! I love what you guys are building. I noticed you are currently running paid ads, but your website takes a massive 28.3 seconds to load. You are paying for traffic but likely losing customers to slow load times before they see your products. I built a high-speed React prototype for you that loads instantly with a 1-click WhatsApp checkout. Check it out here: https://pkgarments-demo.netlify.app/ Let me know what you think!</t>
-  </si>
-  <si>
     <t>screenshots/CANVAS_Salon_Lahore___Best_Hair_and_Bridal_Parlour_Gulberg.png</t>
   </si>
   <si>
@@ -250,9 +227,6 @@
     <t>36.9s</t>
   </si>
   <si>
-    <t>Hello Kashee's Beauty Parlour Lahore team! I love what you guys are building. I noticed you are currently running paid ads, but your website takes a massive 36.9 seconds to load. You are paying for traffic but likely losing customers to slow load times before they see your products. I built a high-speed React prototype for you that loads instantly with a 1-click WhatsApp checkout. Check it out here: https://pkgarments-demo.netlify.app/ Let me know what you think!</t>
-  </si>
-  <si>
     <t>screenshots/Kashee_s_Beauty_Parlour_Lahore.png</t>
   </si>
   <si>
@@ -269,27 +243,61 @@
   </si>
   <si>
     <t>screenshots/Kashi_Beauty_Saloon_ERROR.png</t>
+  </si>
+  <si>
+    <t>Hello Fuzion Salon &amp; Spa team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Kauser beauty parlour team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello 𝐁𝐞𝐚𝐮𝐭𝐲 𝐂𝐚𝐫𝐞 𝐛𝐲 𝐍𝐚𝐛𝐢𝐥𝐚 (Gulberg Branch) team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Beauty Icon Salon, Makeup Lounge &amp; Ladies GYM team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Beauty Queen Beauty Parlour team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Shimla Beauty Parlor - Hair Salon Best beauty parlor in Lahore team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Hamna's Beauty salon &amp; Bridal Studio team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Shafaq n Kami salon | Best Salon &amp; Studio in Lahore, Pakistan team! I love what you guys are building. I noticed you are currently running paid ads, but your website takes a massive 6.8 seconds to load. You are paying for traffic but likely losing customers to slow load times before they see your products. I built a high-speed React prototype for you that loads instantly with a 1-click WhatsApp checkout. Check it out here: https://jalaldev.tech/salon.html Let me know what you think!</t>
+  </si>
+  <si>
+    <t>Hello CANVAS Salon Lahore | Best Hair and Bridal Parlour Gulberg team! I love what you guys are building. I noticed you are currently running paid ads, but your website takes a massive 28.3 seconds to load. You are paying for traffic but likely losing customers to slow load times before they see your products. I built a high-speed React prototype for you that loads instantly with a 1-click WhatsApp checkout. Check it out here: https://jalaldev.tech/salon.html Let me know what you think!</t>
+  </si>
+  <si>
+    <t>Hello Kashee's Beauty Parlour Lahore team! I love what you guys are building. I noticed you are currently running paid ads, but your website takes a massive 36.9 seconds to load. You are paying for traffic but likely losing customers to slow load times before they see your products. I built a high-speed React prototype for you that loads instantly with a 1-click WhatsApp checkout. Check it out here: https://jalaldev.tech/salon.html Let me know what you think!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
       <u/>
+      <sz val="11"/>
       <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -659,9 +667,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -775,7 +783,7 @@
         <v>21</v>
       </c>
       <c r="O2" t="s">
-        <v>22</v>
+        <v>76</v>
       </c>
       <c r="P2" t="s">
         <v>20</v>
@@ -786,10 +794,10 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
         <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>24</v>
       </c>
       <c r="D3" t="s">
         <v>16</v>
@@ -822,10 +830,10 @@
         <v>20</v>
       </c>
       <c r="N3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O3" t="s">
-        <v>25</v>
+        <v>77</v>
       </c>
       <c r="P3" t="s">
         <v>20</v>
@@ -836,10 +844,10 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
         <v>16</v>
@@ -875,7 +883,7 @@
         <v>21</v>
       </c>
       <c r="O4" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="P4" t="s">
         <v>20</v>
@@ -886,10 +894,10 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
@@ -922,10 +930,10 @@
         <v>20</v>
       </c>
       <c r="N5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O5" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="P5" t="s">
         <v>20</v>
@@ -936,10 +944,10 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
         <v>16</v>
@@ -975,7 +983,7 @@
         <v>21</v>
       </c>
       <c r="O6" t="s">
-        <v>33</v>
+        <v>80</v>
       </c>
       <c r="P6" t="s">
         <v>20</v>
@@ -986,10 +994,10 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
         <v>16</v>
@@ -1025,7 +1033,7 @@
         <v>21</v>
       </c>
       <c r="O7" t="s">
-        <v>36</v>
+        <v>81</v>
       </c>
       <c r="P7" t="s">
         <v>20</v>
@@ -1036,10 +1044,10 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D8" t="s">
         <v>16</v>
@@ -1075,7 +1083,7 @@
         <v>21</v>
       </c>
       <c r="O8" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="P8" t="s">
         <v>20</v>
@@ -1083,34 +1091,34 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E9" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="I9" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J9" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="K9">
         <v>200</v>
@@ -1125,42 +1133,42 @@
         <v>21</v>
       </c>
       <c r="O9" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="P9" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E10" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="F10" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G10" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="H10" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="I10" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="J10" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="K10">
         <v>135</v>
@@ -1175,42 +1183,42 @@
         <v>21</v>
       </c>
       <c r="O10" t="s">
-        <v>54</v>
+        <v>83</v>
       </c>
       <c r="P10" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="F11" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G11" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="H11" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="I11" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="J11" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="K11">
         <v>125</v>
@@ -1225,42 +1233,42 @@
         <v>21</v>
       </c>
       <c r="O11" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="P11" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F12" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G12" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="H12" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="I12" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J12" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="K12">
         <v>200</v>
@@ -1275,7 +1283,7 @@
         <v>21</v>
       </c>
       <c r="O12" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="P12" t="s">
         <v>20</v>
@@ -1283,34 +1291,34 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="D13" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E13" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F13" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G13" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="H13" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="I13" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J13" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="K13">
         <v>200</v>
@@ -1325,7 +1333,7 @@
         <v>21</v>
       </c>
       <c r="O13" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="P13" t="s">
         <v>20</v>
@@ -1333,34 +1341,34 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="D14" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="E14" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F14" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G14" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="H14" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="I14" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J14" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="K14">
         <v>200</v>
@@ -1375,42 +1383,42 @@
         <v>21</v>
       </c>
       <c r="O14" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="P14" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="C15" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="D15" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="E15" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="F15" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G15" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="H15" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="I15" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="J15" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="K15">
         <v>130</v>
@@ -1425,42 +1433,42 @@
         <v>21</v>
       </c>
       <c r="O15" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="P15" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="D16" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="E16" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F16" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G16" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="H16" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="I16" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J16" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="K16">
         <v>200</v>
@@ -1475,29 +1483,29 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="P16" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="N2" r:id="rId1"/>
-    <hyperlink ref="N4" r:id="rId2"/>
-    <hyperlink ref="N6" r:id="rId3"/>
-    <hyperlink ref="N7" r:id="rId4"/>
-    <hyperlink ref="N8" r:id="rId5"/>
-    <hyperlink ref="N9" r:id="rId6"/>
-    <hyperlink ref="N10" r:id="rId7"/>
-    <hyperlink ref="N11" r:id="rId8"/>
-    <hyperlink ref="N12" r:id="rId9"/>
-    <hyperlink ref="N13" r:id="rId10"/>
-    <hyperlink ref="N14" r:id="rId11"/>
-    <hyperlink ref="N15" r:id="rId12"/>
-    <hyperlink ref="N16" r:id="rId13"/>
+    <hyperlink ref="N2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="N4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="N6" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="N7" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="N8" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="N9" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N10" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="N11" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="N12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="N13" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="N14" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="N15" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="N16" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added Random Search queery selector
</commit_message>
<xml_diff>
--- a/leads_crm.xlsx
+++ b/leads_crm.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DE4E7AD-C982-4265-9333-D5245272F4A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Qualified Leads" state="visible" r:id="rId4"/>
+    <sheet name="Qualified Leads" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="126">
   <si>
     <t>Category</t>
   </si>
@@ -85,7 +89,7 @@
     <t>Phone: +92 321 3314177</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Zehra+Abbas+PECHS/data=!4m7!3m6!1s0x3eb33f180555dd87:0x84b7a50e4e956c57!8m2!3d24.8688411!4d67.0589013!16s%2Fg%2F11jwzz3sms!19sChIJh91VBRg_sz4RV2yVTg6lt4Q?authuser=0&amp;hl=en&amp;rclk=1</t>
+    <t>https://www.google.com/maps/place/Zehra+Abbas+PECHS/@24.8688411,67.0589013,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33f180555dd87:0x84b7a50e4e956c57!8m2!3d24.8688411!4d67.0589013!16s%2Fg%2F11jwzz3sms?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>N/A</t>
@@ -100,19 +104,13 @@
     <t>📲 Send Message</t>
   </si>
   <si>
-    <t>Hello Zehra Abbas PECHS team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
-  </si>
-  <si>
     <t>Flourish Salon - Aqsa Danish</t>
   </si>
   <si>
     <t>Phone: +92 21 34833323</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Flourish+Salon+-+Aqsa+Danish/data=!4m7!3m6!1s0x3eb33f4a9793b1c7:0xcd24bc4ff3c95b54!8m2!3d24.9277963!4d67.0925359!16s%2Fg%2F11hb5bm7xz!19sChIJx7GTl0o_sz4RVFvJ80-8JM0?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello Flourish Salon - Aqsa Danish team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
+    <t>https://www.google.com/maps/place/Flourish+Salon+-+Aqsa+Danish/@24.9277963,67.0925359,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33f4a9793b1c7:0xcd24bc4ff3c95b54!8m2!3d24.9277963!4d67.0925359!16s%2Fg%2F11hb5bm7xz?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>ivory Salon by Anum Zubair (Gulshan Branch)</t>
@@ -121,10 +119,7 @@
     <t>Phone: +92 345 2345055</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/ivory+Salon+by+Anum+Zubair+%28Gulshan+Branch%29/data=!4m7!3m6!1s0x3eb33fe2d02962fb:0x9e2b22ea3e595fb6!8m2!3d24.9193219!4d67.0853721!16s%2Fg%2F11h84mvb51!19sChIJ-2Ip0OI_sz4Rtl9ZPuoiK54?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello ivory Salon by Anum Zubair (Gulshan Branch) team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
+    <t>https://www.google.com/maps/place/ivory+Salon+by+Anum+Zubair+(Gulshan+Branch)/@24.9193219,67.0853721,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33fe2d02962fb:0x9e2b22ea3e595fb6!8m2!3d24.9193219!4d67.0853721!16s%2Fg%2F11h84mvb51?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>Imperial - Beauty Salon and Spa</t>
@@ -133,10 +128,7 @@
     <t>Phone: +92 333 8748899</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Imperial+-+Beauty+Salon+and+Spa/data=!4m7!3m6!1s0x3eb33909a99afcab:0xf188a07ef281bdde!8m2!3d24.929756!4d67.0974316!16s%2Fg%2F11jht3pvlk!19sChIJq_yaqQk5sz4R3r2B8n6giPE?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello Imperial - Beauty Salon and Spa team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
+    <t>https://www.google.com/maps/place/Imperial+-+Beauty+Salon+and+Spa/@24.929756,67.0974316,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33909a99afcab:0xf188a07ef281bdde!8m2!3d24.929756!4d67.0974316!16s%2Fg%2F11jht3pvlk?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>Zoellas beauty Salon</t>
@@ -145,10 +137,7 @@
     <t>Phone: +92 311 1802834</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Zoellas+beauty+Salon/data=!4m7!3m6!1s0x3eb33e93d2e17e17:0xe2e05f75145dc88e!8m2!3d24.8720831!4d67.0610108!16s%2Fg%2F11bzv34ntc!19sChIJF37h0pM-sz4RjshdFHVf4OI?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello Zoellas beauty Salon team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
+    <t>https://www.google.com/maps/place/Zoellas+beauty+Salon/@24.8720831,67.0610108,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33e93d2e17e17:0xe2e05f75145dc88e!8m2!3d24.8720831!4d67.0610108!16s%2Fg%2F11bzv34ntc?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>AIMS BEAUTY SALON (GULSHAN BRANCH)</t>
@@ -157,10 +146,7 @@
     <t>Phone: +92 333 9368111</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/AIMS+BEAUTY+SALON+%28GULSHAN+BRANCH%29/data=!4m7!3m6!1s0x3eb33f8eba1f5215:0xe013da215dd9c1de!8m2!3d24.9078573!4d67.0745373!16s%2Fg%2F11kqmv4w0l!19sChIJFVIfuo4_sz4R3sHZXSHaE-A?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello AIMS BEAUTY SALON (GULSHAN BRANCH) team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
+    <t>https://www.google.com/maps/place/AIMS+BEAUTY+SALON+(GULSHAN+BRANCH)/@24.9078573,67.0745373,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33f8eba1f5215:0xe013da215dd9c1de!8m2!3d24.9078573!4d67.0745373!16s%2Fg%2F11kqmv4w0l?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>Avenue Salon &amp; Spa</t>
@@ -169,10 +155,7 @@
     <t>Phone: +92 21 34169966</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Avenue+Salon+%26+Spa/data=!4m7!3m6!1s0x3eb33eb66c90e7b1:0x8ec3bd58f6027df4!8m2!3d24.879774!4d67.0870819!16s%2Fg%2F11c3s9583w!19sChIJseeQbLY-sz4R9H0C9li9w44?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello Avenue Salon &amp; Spa team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
+    <t>https://www.google.com/maps/place/Avenue+Salon+%26+Spa/@24.879774,67.0870819,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33eb66c90e7b1:0x8ec3bd58f6027df4!8m2!3d24.879774!4d67.0870819!16s%2Fg%2F11c3s9583w?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>Ivory Salon by Anum Zubair (Nazimabad Branch)</t>
@@ -181,10 +164,7 @@
     <t>Phone: +92 335 2345055</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Ivory+Salon+by+Anum+Zubair+%28Nazimabad+Branch%29/data=!4m7!3m6!1s0x3eb33f323c21a599:0x45678ba93f05d149!8m2!3d24.9194406!4d67.0331985!16s%2Fg%2F11vxv257g4!19sChIJmaUhPDI_sz4RSdEFP6mLZ0U?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello Ivory Salon by Anum Zubair (Nazimabad Branch) team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
+    <t>https://www.google.com/maps/place/Ivory+Salon+by+Anum+Zubair+(Nazimabad+Branch)/@24.9194406,67.0331985,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33f323c21a599:0x45678ba93f05d149!8m2!3d24.9194406!4d67.0331985!16s%2Fg%2F11vxv257g4?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>Najla's Beauty Parlour</t>
@@ -193,10 +173,7 @@
     <t>Phone: +92 21 34385276</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Najla%27s+Beauty+Parlour/data=!4m7!3m6!1s0x3eb33e8e223e52d1:0x339b286ff65ac426!8m2!3d24.8695899!4d67.0579525!16s%2Fg%2F11ggt189hl!19sChIJ0VI-Io4-sz4RJsRa9m8omzM?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello Najla's Beauty Parlour team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
+    <t>https://www.google.com/maps/place/Najla's+Beauty+Parlour/@24.8695899,67.0579525,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33e8e223e52d1:0x339b286ff65ac426!8m2!3d24.8695899!4d67.0579525!16s%2Fg%2F11ggt189hl?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>Somi's Glamour Beauty Salon &amp; Training Center</t>
@@ -205,10 +182,7 @@
     <t>No Phone</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Somi%27s+Glamour+Beauty+Salon+%26+Training+Center/data=!4m7!3m6!1s0x3eb33d1dd67cdd7f:0x6a7323a28f944fcb!8m2!3d24.8534873!4d67.0729221!16s%2Fg%2F11pb7l647k!19sChIJf9181h09sz4Ry0-Uj6Ijc2o?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello Somi's Glamour Beauty Salon &amp; Training Center team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
+    <t>https://www.google.com/maps/place/Somi's+Glamour+Beauty+Salon+%26+Training+Center/@24.8534873,67.0729221,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33d1dd67cdd7f:0x6a7323a28f944fcb!8m2!3d24.8534873!4d67.0729221!16s%2Fg%2F11pb7l647k?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>Najlas Beauty Parlor</t>
@@ -217,10 +191,7 @@
     <t>Phone: +92 336 2542923</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Najlas+Beauty+Parlor/data=!4m7!3m6!1s0x3eb338b54b11f85f:0xe7d742380b23299c!8m2!3d24.9280675!4d67.0946077!16s%2Fg%2F11fzf3x1ww!19sChIJX_gRS7U4sz4RnCkjCzhC1-c?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello Najlas Beauty Parlor team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
+    <t>https://www.google.com/maps/place/Najlas+Beauty+Parlor/@24.9280675,67.0946077,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb338b54b11f85f:0xe7d742380b23299c!8m2!3d24.9280675!4d67.0946077!16s%2Fg%2F11fzf3x1ww?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>Zari's Beauty Parlour</t>
@@ -229,10 +200,7 @@
     <t>Phone: +92 301 2498054</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Zari%27s+Beauty+Parlour/data=!4m7!3m6!1s0x3eb33db5312a712b:0x241a12d466bef81!8m2!3d24.8495846!4d67.0511615!16s%2Fg%2F11twr2rbg1!19sChIJK3EqMbU9sz4Rge9rRi2hQQI?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello Zari's Beauty Parlour team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://pkgarments-demo.netlify.app/ Would you be open to a quick chat?</t>
+    <t>https://www.google.com/maps/place/Zari's+Beauty+Parlour/@24.8495846,67.0511615,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33db5312a712b:0x241a12d466bef81!8m2!3d24.8495846!4d67.0511615!16s%2Fg%2F11twr2rbg1?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>Needs Redesign/Audit</t>
@@ -247,7 +215,7 @@
     <t>https://nabila.net/nabila-clifton-karachi/</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/NABILA+Clifton+Karachi/data=!4m7!3m6!1s0x3eb33d083ee61007:0xded3cbf202960258!8m2!3d24.8044876!4d67.0309225!16s%2Fg%2F1jkvnw3bs!19sChIJBxDmPgg9sz4RWAKWAvLL094?authuser=0&amp;hl=en&amp;rclk=1</t>
+    <t>https://www.google.com/maps/place/NABILA+Clifton+Karachi/@24.8044876,67.0309225,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33d083ee61007:0xded3cbf202960258!8m2!3d24.8044876!4d67.0309225!16s%2Fg%2F1jkvnw3bs?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>⚠️ TIMEOUT</t>
@@ -262,24 +230,6 @@
     <t>screenshots/NABILA_Clifton_Karachi_ERROR.png</t>
   </si>
   <si>
-    <t>Sana Sarah's Salon &amp; Studio - Johar Branch</t>
-  </si>
-  <si>
-    <t>Phone: +92 317 2129212</t>
-  </si>
-  <si>
-    <t>https://sanasarahssalon.com/</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/place/Sana+Sarah%27s+Salon+%26+Studio+-+Johar+Branch/data=!4m7!3m6!1s0x3eb338eef9fd9b55:0xeee23238f2d49f0c!8m2!3d24.9249041!4d67.126441!16s%2Fg%2F11csqh111j!19sChIJVZv9-e44sz4RDJ_U8jgy4u4?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>Hello Sana Sarah's Salon &amp; Studio - Johar Branch team! I was just trying to check out your products/services, but your website is currently down and throwing an error page. You are likely losing traffic and buyers right now. I build high-speed, secure React stores with 1-click WhatsApp checkout. Would you like me to help get your digital storefront back online quickly?</t>
-  </si>
-  <si>
-    <t>screenshots/Sana_Sarah_s_Salon___Studio___Johar_Branch_ERROR.png</t>
-  </si>
-  <si>
     <t>Rejuve Luxury Salon &amp; Spa</t>
   </si>
   <si>
@@ -289,7 +239,7 @@
     <t>https://www.rejuvebyaliyafarooq.com/</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Rejuve+Luxury+Salon+%26+Spa/data=!4m7!3m6!1s0x3eb33eb614c79b89:0xc46226ca4e0d2b04!8m2!3d24.8801008!4d67.0868264!16s%2Fg%2F11hbk48lhj!19sChIJiZvHFLY-sz4RBCsNTsomYsQ?authuser=0&amp;hl=en&amp;rclk=1</t>
+    <t>https://www.google.com/maps/place/Rejuve+Luxury+Salon+%26+Spa/@24.8801008,67.0868264,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33eb614c79b89:0xc46226ca4e0d2b04!8m2!3d24.8801008!4d67.0868264!16s%2Fg%2F11hbk48lhj?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>Hello Rejuve Luxury Salon &amp; Spa team! I was just trying to check out your products/services, but your website is currently down and throwing an error page. You are likely losing traffic and buyers right now. I build high-speed, secure React stores with 1-click WhatsApp checkout. Would you like me to help get your digital storefront back online quickly?</t>
@@ -307,10 +257,10 @@
     <t>https://kashees.com/</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Kashee%27s+Beauty+Parlour/data=!4m7!3m6!1s0x3eb33e8fb8859653:0x22f69c58064e603b!8m2!3d24.8674281!4d67.0574319!16s%2Fg%2F11c5zy03xk!19sChIJU5aFuI8-sz4RO2BOBlic9iI?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>11.2s</t>
+    <t>https://www.google.com/maps/place/Kashee's+Beauty+Parlour/@24.8674281,67.0574319,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33e8fb8859653:0x22f69c58064e603b!8m2!3d24.8674281!4d67.0574319!16s%2Fg%2F11c5zy03xk?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>11.6s</t>
   </si>
   <si>
     <t>✅ Yes</t>
@@ -328,34 +278,31 @@
     <t>{"facebook":"https://www.facebook.com/kasheesbeautyparlor","instagram":"https://www.instagram.com/kashees_official","linkedin":"None","tiktok":"https://www.tiktok.com/@kashees.official"}</t>
   </si>
   <si>
-    <t>Hello Kashee's Beauty Parlour team! I love what you guys are building. I noticed you are currently running paid ads, but your website takes a massive 11.2 seconds to load. You are paying for traffic but likely losing customers to slow load times before they see your products. I built a high-speed React prototype for you that loads instantly with a 1-click WhatsApp checkout. Check it out here: https://pkgarments-demo.netlify.app/ Let me know what you think!</t>
-  </si>
-  <si>
     <t>screenshots/Kashee_s_Beauty_Parlour.png</t>
   </si>
   <si>
-    <t>Najla's Beauty Salon &amp; Spa - Tariq Road Branch</t>
-  </si>
-  <si>
-    <t>Phone: +92 337 2429641</t>
-  </si>
-  <si>
-    <t>https://najlasbeautyclinic.com/</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/place/Najla%27s+Beauty+Salon+%26+Spa+-+Tariq+Road+Branch/data=!4m7!3m6!1s0x3eb33fae903e5bcb:0x4a36a2a2eeb2d5c!8m2!3d24.8787345!4d67.0643958!16s%2Fg%2F11x0qbvs_m!19sChIJy1s-kK4_sz4RXC3rLipqowQ?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>6.8s</t>
-  </si>
-  <si>
-    <t>{"facebook":"None","instagram":"None","linkedin":"None","tiktok":"None"}</t>
-  </si>
-  <si>
-    <t>Hello Najla's Beauty Salon &amp; Spa - Tariq Road Branch team! I love what you guys are building. I did a quick performance test and noticed your website takes 6.8 seconds to load. Amazon found that every 1 second of delay costs 7% in sales. I built a high-speed React prototype for you with a 1-click WhatsApp checkout to fix this. Check it out here: https://pkgarments-demo.netlify.app/ Let me know what you think!</t>
-  </si>
-  <si>
-    <t>screenshots/Najla_s_Beauty_Salon___Spa___Tariq_Road_Branch.png</t>
+    <t>Lavish Women Salon Johar Branch</t>
+  </si>
+  <si>
+    <t>Phone: +92 336 4440129</t>
+  </si>
+  <si>
+    <t>https://lavishsaloon.com.pk/</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Lavish+Women+Salon+Johar+Branch/@24.9312461,67.1391375,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb339acaac4036f:0xf30390dc10d1a8b2!8m2!3d24.9312461!4d67.1391375!16s%2Fg%2F11ts4c4yh4?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>7.3s</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/lavishmensalon/ | https://www.instagram.com/lavishmensalon/</t>
+  </si>
+  <si>
+    <t>{"facebook":"https://www.facebook.com/lavishmensalon/","instagram":"https://www.instagram.com/lavishmensalon/","linkedin":"None","tiktok":"None"}</t>
+  </si>
+  <si>
+    <t>screenshots/Lavish_Women_Salon_Johar_Branch.png</t>
   </si>
   <si>
     <t>Gillan Salon &amp; Spa</t>
@@ -367,7 +314,7 @@
     <t>http://www.gillan.pk/</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Gillan+Salon+%26+Spa/data=!4m7!3m6!1s0x3eb33cf272762da9:0xaee7abdc911ff74e!8m2!3d24.8001811!4d67.0662865!16s%2Fg%2F1hc2_8m8h!19sChIJqS12cvI8sz4RTvcfkdyr564?authuser=0&amp;hl=en&amp;rclk=1</t>
+    <t>https://www.google.com/maps/place/Gillan+Salon+%26+Spa/@24.8001811,67.0662865,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb33cf272762da9:0xaee7abdc911ff74e!8m2!3d24.8001811!4d67.0662865!16s%2Fg%2F1hc2_8m8h?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
     <t>Hello Gillan Salon &amp; Spa team! I was just trying to check out your products/services, but your website is currently down and throwing an error page. You are likely losing traffic and buyers right now. I build high-speed, secure React stores with 1-click WhatsApp checkout. Would you like me to help get your digital storefront back online quickly?</t>
@@ -385,10 +332,10 @@
     <t>http://enhancebsalon.com/</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Enhance+beauty+salon/data=!4m7!3m6!1s0x3eb341175a3d85c1:0x399cced7984c3da5!8m2!3d24.9724195!4d67.064315!16s%2Fg%2F11j0tvr88t!19sChIJwYU9WhdBsz4RpT1MmNfOnDk?authuser=0&amp;hl=en&amp;rclk=1</t>
-  </si>
-  <si>
-    <t>21.8s</t>
+    <t>https://www.google.com/maps/place/Enhance+beauty+salon/@24.9724195,67.064315,17z/data=!3m1!4b1!4m6!3m5!1s0x3eb341175a3d85c1:0x399cced7984c3da5!8m2!3d24.9724195!4d67.064315!16s%2Fg%2F11j0tvr88t?authuser=0&amp;hl=en&amp;entry=ttu&amp;g_ep=EgoyMDI2MDYyNC4wIKXMDSoASAFQAw%3D%3D</t>
+  </si>
+  <si>
+    <t>10.8s</t>
   </si>
   <si>
     <t>info@enhancebsalon.com</t>
@@ -400,31 +347,85 @@
     <t>{"facebook":"https://www.facebook.com/asmaqaiyum1/","instagram":"https://www.instagram.com/enhancebeautysalon39/","linkedin":"None","tiktok":"None"}</t>
   </si>
   <si>
-    <t>Hello Enhance beauty salon team! I love what you guys are building. I did a quick performance test and noticed your website takes 21.8 seconds to load. Amazon found that every 1 second of delay costs 7% in sales. I built a high-speed React prototype for you with a 1-click WhatsApp checkout to fix this. Check it out here: https://pkgarments-demo.netlify.app/ Let me know what you think!</t>
-  </si>
-  <si>
     <t>screenshots/Enhance_beauty_salon.png</t>
+  </si>
+  <si>
+    <t>Hello Zehra Abbas PECHS team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Flourish Salon - Aqsa Danish team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello ivory Salon by Anum Zubair (Gulshan Branch) team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Imperial - Beauty Salon and Spa team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Zoellas beauty Salon team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello AIMS BEAUTY SALON (GULSHAN BRANCH) team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Avenue Salon &amp; Spa team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Ivory Salon by Anum Zubair (Nazimabad Branch) team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Najla's Beauty Parlour team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Somi's Glamour Beauty Salon &amp; Training Center team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Najlas Beauty Parlor team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Zari's Beauty Parlour team! I noticed you are running a great brand in Lahore but don't have a dedicated website yet. I build custom React online stores that connect directly to WhatsApp for easy ordering. I built a live demo so you can see how it works: https://jalaldev.tech/salon.html Would you be open to a quick chat?</t>
+  </si>
+  <si>
+    <t>Hello Kashee's Beauty Parlour team! Your premium collection truly elevates natural beauty. I noticed you are currently running paid ads, but your website takes a massive 11.6 seconds to load. You are paying for traffic but likely losing customers to slow load times before they see your products. I built a high-speed React prototype for you that loads instantly with a 1-click WhatsApp checkout. Check it out here: https://jalaldev.tech/salon.html Let me know what you think!</t>
+  </si>
+  <si>
+    <t>Hello Lavish Women Salon Johar Branch team! Your salon’s vibe is pure luxury, love the Johar spot! I noticed you are currently running paid ads, but your website takes a massive 7.3 seconds to load. You are paying for traffic but likely losing customers to slow load times before they see your products. I built a high-speed React prototype for you that loads instantly with a 1-click WhatsApp checkout. Check it out here: https://jalaldev.tech/salon.html Let me know what you think!</t>
+  </si>
+  <si>
+    <t>Hello Enhance beauty salon team! Your diverse beauty services deserve a fresh, modern online presence. I did a quick performance test and noticed your website takes 10.8 seconds to load. Amazon found that every 1 second of delay costs 7% in sales. I built a high-speed React prototype for you with a 1-click WhatsApp checkout to fix this. Check it out here: https://jalaldev.tech/salon.html Let me know what you think!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <color rgb="FF0563C1"/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -449,15 +450,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -794,9 +798,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U20"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:U19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -897,7 +901,7 @@
       <c r="D2" t="s">
         <v>21</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F2" t="s">
@@ -943,7 +947,7 @@
         <v>28</v>
       </c>
       <c r="T2" t="s">
-        <v>29</v>
+        <v>111</v>
       </c>
       <c r="U2" t="s">
         <v>26</v>
@@ -954,16 +958,16 @@
         <v>21</v>
       </c>
       <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
         <v>30</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="D3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" t="s">
-        <v>32</v>
       </c>
       <c r="F3" t="s">
         <v>25</v>
@@ -1008,7 +1012,7 @@
         <v>28</v>
       </c>
       <c r="T3" t="s">
-        <v>33</v>
+        <v>112</v>
       </c>
       <c r="U3" t="s">
         <v>26</v>
@@ -1019,16 +1023,16 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="C4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>36</v>
       </c>
       <c r="F4" t="s">
         <v>25</v>
@@ -1073,7 +1077,7 @@
         <v>28</v>
       </c>
       <c r="T4" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="U4" t="s">
         <v>26</v>
@@ -1084,16 +1088,16 @@
         <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
         <v>21</v>
       </c>
-      <c r="E5" t="s">
-        <v>40</v>
+      <c r="E5" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="F5" t="s">
         <v>25</v>
@@ -1138,7 +1142,7 @@
         <v>28</v>
       </c>
       <c r="T5" t="s">
-        <v>41</v>
+        <v>114</v>
       </c>
       <c r="U5" t="s">
         <v>26</v>
@@ -1149,16 +1153,16 @@
         <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
         <v>21</v>
       </c>
-      <c r="E6" t="s">
-        <v>44</v>
+      <c r="E6" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="F6" t="s">
         <v>25</v>
@@ -1203,7 +1207,7 @@
         <v>28</v>
       </c>
       <c r="T6" t="s">
-        <v>45</v>
+        <v>115</v>
       </c>
       <c r="U6" t="s">
         <v>26</v>
@@ -1214,16 +1218,16 @@
         <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
         <v>21</v>
       </c>
-      <c r="E7" t="s">
-        <v>48</v>
+      <c r="E7" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="F7" t="s">
         <v>25</v>
@@ -1268,7 +1272,7 @@
         <v>28</v>
       </c>
       <c r="T7" t="s">
-        <v>49</v>
+        <v>116</v>
       </c>
       <c r="U7" t="s">
         <v>26</v>
@@ -1279,16 +1283,16 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D8" t="s">
         <v>21</v>
       </c>
-      <c r="E8" t="s">
-        <v>52</v>
+      <c r="E8" s="2" t="s">
+        <v>46</v>
       </c>
       <c r="F8" t="s">
         <v>25</v>
@@ -1333,7 +1337,7 @@
         <v>28</v>
       </c>
       <c r="T8" t="s">
-        <v>53</v>
+        <v>117</v>
       </c>
       <c r="U8" t="s">
         <v>26</v>
@@ -1344,16 +1348,16 @@
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
         <v>21</v>
       </c>
-      <c r="E9" t="s">
-        <v>56</v>
+      <c r="E9" s="2" t="s">
+        <v>49</v>
       </c>
       <c r="F9" t="s">
         <v>25</v>
@@ -1398,7 +1402,7 @@
         <v>28</v>
       </c>
       <c r="T9" t="s">
-        <v>57</v>
+        <v>118</v>
       </c>
       <c r="U9" t="s">
         <v>26</v>
@@ -1409,16 +1413,16 @@
         <v>21</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C10" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
       </c>
-      <c r="E10" t="s">
-        <v>60</v>
+      <c r="E10" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="F10" t="s">
         <v>25</v>
@@ -1463,7 +1467,7 @@
         <v>28</v>
       </c>
       <c r="T10" t="s">
-        <v>61</v>
+        <v>119</v>
       </c>
       <c r="U10" t="s">
         <v>26</v>
@@ -1474,16 +1478,16 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="D11" t="s">
         <v>21</v>
       </c>
-      <c r="E11" t="s">
-        <v>64</v>
+      <c r="E11" s="2" t="s">
+        <v>55</v>
       </c>
       <c r="F11" t="s">
         <v>25</v>
@@ -1525,10 +1529,10 @@
         <v>26</v>
       </c>
       <c r="S11" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="T11" t="s">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="U11" t="s">
         <v>26</v>
@@ -1539,16 +1543,16 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="D12" t="s">
         <v>21</v>
       </c>
-      <c r="E12" t="s">
-        <v>68</v>
+      <c r="E12" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="F12" t="s">
         <v>25</v>
@@ -1593,7 +1597,7 @@
         <v>28</v>
       </c>
       <c r="T12" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
       <c r="U12" t="s">
         <v>26</v>
@@ -1604,16 +1608,16 @@
         <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="D13" t="s">
         <v>21</v>
       </c>
-      <c r="E13" t="s">
-        <v>72</v>
+      <c r="E13" s="2" t="s">
+        <v>61</v>
       </c>
       <c r="F13" t="s">
         <v>25</v>
@@ -1658,7 +1662,7 @@
         <v>28</v>
       </c>
       <c r="T13" t="s">
-        <v>73</v>
+        <v>122</v>
       </c>
       <c r="U13" t="s">
         <v>26</v>
@@ -1666,37 +1670,37 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C14" t="s">
-        <v>76</v>
-      </c>
-      <c r="D14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E14" t="s">
-        <v>78</v>
+        <v>64</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>66</v>
       </c>
       <c r="F14" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="G14" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="H14" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="I14" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="J14" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="K14" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="L14">
         <v>200</v>
@@ -1723,45 +1727,45 @@
         <v>28</v>
       </c>
       <c r="T14" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="U14" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B15" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B15" t="s">
-        <v>83</v>
-      </c>
-      <c r="C15" t="s">
-        <v>84</v>
-      </c>
-      <c r="D15" t="s">
-        <v>85</v>
-      </c>
-      <c r="E15" t="s">
-        <v>86</v>
-      </c>
       <c r="F15" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="G15" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="H15" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="I15" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="J15" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="K15" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="L15">
         <v>200</v>
@@ -1788,110 +1792,110 @@
         <v>28</v>
       </c>
       <c r="T15" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="U15" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B16" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="C16" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="D16" t="s">
-        <v>91</v>
-      </c>
-      <c r="E16" t="s">
-        <v>92</v>
+        <v>79</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>80</v>
       </c>
       <c r="F16" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I16" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="J16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L16">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="M16" t="s">
         <v>26</v>
       </c>
       <c r="N16" t="s">
-        <v>26</v>
+        <v>84</v>
       </c>
       <c r="O16" t="s">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="P16" t="s">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="Q16" t="s">
         <v>27</v>
       </c>
       <c r="R16" t="s">
-        <v>26</v>
+        <v>86</v>
       </c>
       <c r="S16" s="2" t="s">
         <v>28</v>
       </c>
       <c r="T16" t="s">
-        <v>93</v>
+        <v>123</v>
       </c>
       <c r="U16" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B17" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="D17" t="s">
-        <v>97</v>
-      </c>
-      <c r="E17" t="s">
-        <v>98</v>
+        <v>90</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="F17" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="G17" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="H17" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="I17" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="J17" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="K17" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="L17">
         <v>130</v>
@@ -1900,66 +1904,66 @@
         <v>26</v>
       </c>
       <c r="N17" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="O17" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="P17" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="Q17" t="s">
         <v>27</v>
       </c>
       <c r="R17" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="S17" s="2" t="s">
         <v>28</v>
       </c>
       <c r="T17" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="U17" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B18" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C18" t="s">
-        <v>108</v>
-      </c>
-      <c r="D18" t="s">
-        <v>109</v>
-      </c>
-      <c r="E18" t="s">
-        <v>110</v>
+        <v>97</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>99</v>
       </c>
       <c r="F18" t="s">
-        <v>111</v>
+        <v>67</v>
       </c>
       <c r="G18" t="s">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="H18" t="s">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="I18" t="s">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="J18" t="s">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="K18" t="s">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="L18">
-        <v>25</v>
+        <v>200</v>
       </c>
       <c r="M18" t="s">
         <v>26</v>
@@ -1977,170 +1981,125 @@
         <v>27</v>
       </c>
       <c r="R18" t="s">
-        <v>112</v>
+        <v>26</v>
       </c>
       <c r="S18" s="2" t="s">
         <v>28</v>
       </c>
       <c r="T18" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="U18" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="C19" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
       <c r="D19" t="s">
-        <v>117</v>
-      </c>
-      <c r="E19" t="s">
-        <v>118</v>
+        <v>104</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>105</v>
       </c>
       <c r="F19" t="s">
-        <v>79</v>
+        <v>106</v>
       </c>
       <c r="G19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I19" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="J19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="K19" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="L19">
-        <v>200</v>
+        <v>35</v>
       </c>
       <c r="M19" t="s">
-        <v>26</v>
+        <v>107</v>
       </c>
       <c r="N19" t="s">
-        <v>26</v>
+        <v>108</v>
       </c>
       <c r="O19" t="s">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="P19" t="s">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="Q19" t="s">
         <v>27</v>
       </c>
       <c r="R19" t="s">
-        <v>26</v>
+        <v>109</v>
       </c>
       <c r="S19" s="2" t="s">
         <v>28</v>
       </c>
       <c r="T19" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="U19" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>74</v>
-      </c>
-      <c r="B20" t="s">
-        <v>121</v>
-      </c>
-      <c r="C20" t="s">
-        <v>122</v>
-      </c>
-      <c r="D20" t="s">
-        <v>123</v>
-      </c>
-      <c r="E20" t="s">
-        <v>124</v>
-      </c>
-      <c r="F20" t="s">
-        <v>125</v>
-      </c>
-      <c r="G20" t="s">
-        <v>100</v>
-      </c>
-      <c r="H20" t="s">
-        <v>100</v>
-      </c>
-      <c r="I20" t="s">
-        <v>101</v>
-      </c>
-      <c r="J20" t="s">
-        <v>100</v>
-      </c>
-      <c r="K20" t="s">
-        <v>101</v>
-      </c>
-      <c r="L20">
-        <v>35</v>
-      </c>
-      <c r="M20" t="s">
-        <v>126</v>
-      </c>
-      <c r="N20" t="s">
-        <v>127</v>
-      </c>
-      <c r="O20" t="s">
-        <v>103</v>
-      </c>
-      <c r="P20" t="s">
-        <v>103</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>27</v>
-      </c>
-      <c r="R20" t="s">
-        <v>128</v>
-      </c>
-      <c r="S20" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="T20" t="s">
-        <v>129</v>
-      </c>
-      <c r="U20" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="S2" r:id="rId1"/>
-    <hyperlink ref="S3" r:id="rId2"/>
-    <hyperlink ref="S4" r:id="rId3"/>
-    <hyperlink ref="S5" r:id="rId4"/>
-    <hyperlink ref="S6" r:id="rId5"/>
-    <hyperlink ref="S7" r:id="rId6"/>
-    <hyperlink ref="S8" r:id="rId7"/>
-    <hyperlink ref="S9" r:id="rId8"/>
-    <hyperlink ref="S10" r:id="rId9"/>
-    <hyperlink ref="S12" r:id="rId10"/>
-    <hyperlink ref="S13" r:id="rId11"/>
-    <hyperlink ref="S14" r:id="rId12"/>
-    <hyperlink ref="S15" r:id="rId13"/>
-    <hyperlink ref="S16" r:id="rId14"/>
-    <hyperlink ref="S17" r:id="rId15"/>
-    <hyperlink ref="S18" r:id="rId16"/>
-    <hyperlink ref="S19" r:id="rId17"/>
-    <hyperlink ref="S20" r:id="rId18"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="S2" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E3" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="S3" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="E4" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="S4" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="E5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="S5" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="E6" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="S6" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="E7" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="S7" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="E8" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="S8" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="E9" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="S9" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="E10" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="S10" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="E11" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="E12" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="S12" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="E13" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="S13" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="E14" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="S14" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="E15" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="S15" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="E16" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="S16" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="E17" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="S17" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="E18" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="S18" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="E19" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="S19" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="D15" r:id="rId36" xr:uid="{D5C67365-8401-443D-9A9A-09180F16AF3A}"/>
+    <hyperlink ref="D18" r:id="rId37" xr:uid="{81F2B5D6-61DD-429D-8089-0E6F17023367}"/>
+    <hyperlink ref="D14" r:id="rId38" xr:uid="{2931DFAF-8A42-4683-AF9E-A2D5662CADAD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>